<commit_message>
include vendor with collab PRs
</commit_message>
<xml_diff>
--- a/vendor/ironcalc/xlsx/tests/calc_tests/DATE_AND_TIME/EOMONTH.xlsx
+++ b/vendor/ironcalc/xlsx/tests/calc_tests/DATE_AND_TIME/EOMONTH.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicolas/Library/CloudStorage/Dropbox/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\elsa\IronCalc\xlsx\tests\calc_tests\DATE_AND_TIME\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{457D9B5E-D067-074F-A1B9-372600254E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5184BBC-FA96-4187-AD23-22DF254FE9F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{09282B2C-36F5-CB4F-AB93-8D5F0BC0AD25}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{09282B2C-36F5-CB4F-AB93-8D5F0BC0AD25}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
   <si>
     <t>date</t>
   </si>
@@ -48,6 +48,126 @@
   </si>
   <si>
     <t>EOMONTH</t>
+  </si>
+  <si>
+    <t>Start on last day of a 31-day month</t>
+  </si>
+  <si>
+    <t>Start on first day of the month</t>
+  </si>
+  <si>
+    <t>Start mid-month</t>
+  </si>
+  <si>
+    <t>Start on a leap day</t>
+  </si>
+  <si>
+    <t>Leap day plus twelve months</t>
+  </si>
+  <si>
+    <t>31-day month into February, leap year</t>
+  </si>
+  <si>
+    <t>31-day month into February, non-leap year</t>
+  </si>
+  <si>
+    <t>31-day month back into February</t>
+  </si>
+  <si>
+    <t>Crossing the year boundary forward</t>
+  </si>
+  <si>
+    <t>Crossing the year boundary backward</t>
+  </si>
+  <si>
+    <t>Maximum date, zero offset</t>
+  </si>
+  <si>
+    <t>Maximum date stepped back one month</t>
+  </si>
+  <si>
+    <t>Maximum serial as a raw number</t>
+  </si>
+  <si>
+    <t>Serial beyond the maximum date</t>
+  </si>
+  <si>
+    <t>Negative date serial</t>
+  </si>
+  <si>
+    <t>Months fraction just under one</t>
+  </si>
+  <si>
+    <t>Months fraction just above minus one</t>
+  </si>
+  <si>
+    <t>Months extremely small positive</t>
+  </si>
+  <si>
+    <t>Months extremely small negative</t>
+  </si>
+  <si>
+    <t>Months at the half-month midpoint</t>
+  </si>
+  <si>
+    <t>Negative months at the midpoint</t>
+  </si>
+  <si>
+    <t>abc</t>
+  </si>
+  <si>
+    <t>Months as non-numeric text</t>
+  </si>
+  <si>
+    <t>-3</t>
+  </si>
+  <si>
+    <t>Months as negative numeric text</t>
+  </si>
+  <si>
+    <t>3.7</t>
+  </si>
+  <si>
+    <t>Months as fractional numeric text</t>
+  </si>
+  <si>
+    <t>Date as non-numeric text</t>
+  </si>
+  <si>
+    <t>2025-06-15</t>
+  </si>
+  <si>
+    <t>Date as an ISO text string</t>
+  </si>
+  <si>
+    <t>44987</t>
+  </si>
+  <si>
+    <t>Date as numeric text</t>
+  </si>
+  <si>
+    <t>Date as boolean TRUE</t>
+  </si>
+  <si>
+    <t>Error propagation in date</t>
+  </si>
+  <si>
+    <t>Error propagation in months</t>
+  </si>
+  <si>
+    <t>Error propagation, #N/A in date</t>
+  </si>
+  <si>
+    <t>Date with a near-full-day time fraction</t>
+  </si>
+  <si>
+    <t>Date with a half-day time fraction</t>
+  </si>
+  <si>
+    <t>Blank month</t>
+  </si>
+  <si>
+    <t>Omitted month</t>
   </si>
 </sst>
 </file>
@@ -120,12 +240,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
@@ -145,9 +266,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -185,7 +306,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -291,7 +412,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -433,18 +554,44 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{A5203647-3D43-4DB4-950C-20CC422BBD3F}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;cc8f9887-f038-4cb4-9c52-91ef65ffc499&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C8670CE-DBF1-894F-A22B-7BE08F7CB20D}">
-  <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F57"/>
+  <sheetFormatPr defaultColWidth="10.6875" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <cols>
+    <col min="1" max="1" width="11.5625" customWidth="1"/>
+    <col min="4" max="4" width="39.3125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -454,9 +601,11 @@
       <c r="C1" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="F1"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A2" s="1">
+        <f t="shared" ref="A2:A16" si="0">DATE(2023,3,2)</f>
         <v>44987</v>
       </c>
       <c r="B2">
@@ -467,226 +616,794 @@
         <v>45230</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A3" s="1">
+        <f t="shared" si="0"/>
         <v>44987</v>
       </c>
       <c r="B3">
         <v>3</v>
       </c>
       <c r="C3" s="4">
-        <f t="shared" ref="C3:C21" si="0">EOMONTH(A3,B3)</f>
+        <f t="shared" ref="C3:C21" si="1">EOMONTH(A3,B3)</f>
         <v>45107</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.5">
       <c r="A4" s="1">
+        <f t="shared" si="0"/>
         <v>44987</v>
       </c>
       <c r="B4">
         <v>-7</v>
       </c>
       <c r="C4" s="4">
+        <f t="shared" si="1"/>
+        <v>44804</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A5" s="1">
         <f t="shared" si="0"/>
-        <v>44804</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
         <v>44987</v>
       </c>
       <c r="B5">
         <v>-123</v>
       </c>
       <c r="C5" s="4">
+        <f t="shared" si="1"/>
+        <v>41274</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A6" s="1">
         <f t="shared" si="0"/>
-        <v>41274</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
         <v>44987</v>
       </c>
       <c r="B6">
         <v>123</v>
       </c>
       <c r="C6" s="4">
+        <f t="shared" si="1"/>
+        <v>48760</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A7" s="1">
         <f t="shared" si="0"/>
-        <v>48760</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
         <v>44987</v>
       </c>
       <c r="B7">
         <v>4.5</v>
       </c>
       <c r="C7" s="4">
+        <f t="shared" si="1"/>
+        <v>45138</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A8" s="1">
         <f t="shared" si="0"/>
-        <v>45138</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
         <v>44987</v>
       </c>
       <c r="B8">
         <v>-4.7</v>
       </c>
       <c r="C8" s="4">
+        <f t="shared" si="1"/>
+        <v>44895</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A9" s="1">
         <f t="shared" si="0"/>
-        <v>44895</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
         <v>44987</v>
       </c>
       <c r="B9">
         <v>-4.2</v>
       </c>
       <c r="C9" s="4">
+        <f t="shared" si="1"/>
+        <v>44895</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A10" s="1">
         <f t="shared" si="0"/>
-        <v>44895</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
         <v>44987</v>
       </c>
       <c r="B10">
         <v>77.8</v>
       </c>
       <c r="C10" s="4">
+        <f t="shared" si="1"/>
+        <v>47361</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A11" s="1">
         <f t="shared" si="0"/>
-        <v>47361</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
         <v>44987</v>
       </c>
       <c r="B11" t="b">
         <v>1</v>
       </c>
       <c r="C11" s="4" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A12" s="1">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
         <v>44987</v>
       </c>
       <c r="B12" t="b">
         <v>0</v>
       </c>
       <c r="C12" s="4" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A13" s="1">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
         <v>44987</v>
       </c>
       <c r="B13">
         <v>0</v>
       </c>
       <c r="C13" s="4">
+        <f t="shared" si="1"/>
+        <v>45016</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A14" s="1">
         <f t="shared" si="0"/>
+        <v>44987</v>
+      </c>
+      <c r="C14" s="4">
+        <f t="shared" si="1"/>
         <v>45016</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>44987</v>
-      </c>
-      <c r="C14" s="4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A15" s="1">
         <f t="shared" si="0"/>
-        <v>45016</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
         <v>44987</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C15" s="4">
+        <f t="shared" si="1"/>
+        <v>45077</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.5">
+      <c r="A16" s="1">
         <f t="shared" si="0"/>
-        <v>45077</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
         <v>44987</v>
       </c>
       <c r="C16" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>45016</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A17" s="1">
+        <f>DATE(1957,3,2)</f>
         <v>20881</v>
       </c>
       <c r="B17">
         <v>1230</v>
       </c>
       <c r="C17" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>58348</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A18" s="1">
+        <f>DATE(2023,3,2)</f>
         <v>44987</v>
       </c>
       <c r="B18">
         <v>-1240.3330000000001</v>
       </c>
       <c r="C18" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7274</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A19" s="1">
+        <f>DATE(2023,11,1)</f>
         <v>45231</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>45291</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A20" s="1">
+        <f>DATE(2023,11,30)</f>
         <v>45260</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>45291</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.5">
       <c r="A21" s="1">
+        <f>DATE(2023,11,1)</f>
         <v>45231</v>
       </c>
       <c r="B21">
         <v>2</v>
       </c>
       <c r="C21" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>45322</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A23" s="1">
+        <f>DATE(2025,1,31)</f>
+        <v>45688</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23" s="4">
+        <f t="shared" ref="C23:C43" si="2">EOMONTH(A23,B23)</f>
+        <v>45688</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A24" s="1">
+        <f>DATE(2025,1,1)</f>
+        <v>45658</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="C24" s="4">
+        <f t="shared" si="2"/>
+        <v>45688</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A25" s="1">
+        <f>DATE(2025,1,15)</f>
+        <v>45672</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="C25" s="4">
+        <f t="shared" si="2"/>
+        <v>45688</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A26" s="1">
+        <f>DATE(2024,2,29)</f>
+        <v>45351</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+      <c r="C26" s="4">
+        <f t="shared" si="2"/>
+        <v>45351</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A27" s="1">
+        <f>DATE(2024,2,29)</f>
+        <v>45351</v>
+      </c>
+      <c r="B27">
+        <v>12</v>
+      </c>
+      <c r="C27" s="4">
+        <f t="shared" si="2"/>
+        <v>45716</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A28" s="1">
+        <f>DATE(2024,1,31)</f>
+        <v>45322</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28" s="4">
+        <f t="shared" si="2"/>
+        <v>45351</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A29" s="1">
+        <f>DATE(2025,1,31)</f>
+        <v>45688</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29" s="4">
+        <f t="shared" si="2"/>
+        <v>45716</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A30" s="1">
+        <f>DATE(2025,3,31)</f>
+        <v>45747</v>
+      </c>
+      <c r="B30">
+        <v>-1</v>
+      </c>
+      <c r="C30" s="4">
+        <f t="shared" si="2"/>
+        <v>45716</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A31" s="1">
+        <f>DATE(2025,12,31)</f>
+        <v>46022</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" s="4">
+        <f t="shared" si="2"/>
+        <v>46053</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A32" s="1">
+        <f>DATE(2025,1,1)</f>
+        <v>45658</v>
+      </c>
+      <c r="B32">
+        <v>-1</v>
+      </c>
+      <c r="C32" s="4">
+        <f t="shared" si="2"/>
+        <v>45657</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A33" s="1">
+        <f>DATE(9999,12,31)</f>
+        <v>2958465</v>
+      </c>
+      <c r="B33">
+        <v>0</v>
+      </c>
+      <c r="C33" s="4">
+        <f t="shared" si="2"/>
+        <v>2958465</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A34" s="1">
+        <f>DATE(9999,12,31)</f>
+        <v>2958465</v>
+      </c>
+      <c r="B34">
+        <v>-1</v>
+      </c>
+      <c r="C34" s="4">
+        <f t="shared" si="2"/>
+        <v>2958434</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A35" s="1">
+        <f>DATE(9999,12,31)</f>
+        <v>2958465</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="C35" s="4">
+        <f t="shared" si="2"/>
+        <v>2958465</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A36">
+        <v>2958466</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36" s="4" t="e">
+        <f t="shared" si="2"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A37">
+        <v>-1</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" s="4" t="e">
+        <f t="shared" si="2"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A38" s="1">
+        <f t="shared" ref="A38:A46" si="3">DATE(2023,3,2)</f>
+        <v>44987</v>
+      </c>
+      <c r="B38">
+        <v>0.99999990000000005</v>
+      </c>
+      <c r="C38" s="4">
+        <f t="shared" si="2"/>
+        <v>45016</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A39" s="1">
+        <f t="shared" si="3"/>
+        <v>44987</v>
+      </c>
+      <c r="B39">
+        <v>-0.99999990000000005</v>
+      </c>
+      <c r="C39" s="4">
+        <f t="shared" si="2"/>
+        <v>45016</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A40" s="1">
+        <f t="shared" si="3"/>
+        <v>44987</v>
+      </c>
+      <c r="B40">
+        <v>9.9999999999999995E-8</v>
+      </c>
+      <c r="C40" s="4">
+        <f t="shared" si="2"/>
+        <v>45016</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A41" s="1">
+        <f t="shared" si="3"/>
+        <v>44987</v>
+      </c>
+      <c r="B41">
+        <v>-9.9999999999999995E-8</v>
+      </c>
+      <c r="C41" s="4">
+        <f t="shared" si="2"/>
+        <v>45016</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A42" s="1">
+        <f t="shared" si="3"/>
+        <v>44987</v>
+      </c>
+      <c r="B42">
+        <v>0.5</v>
+      </c>
+      <c r="C42" s="4">
+        <f t="shared" si="2"/>
+        <v>45016</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A43" s="1">
+        <f t="shared" si="3"/>
+        <v>44987</v>
+      </c>
+      <c r="B43">
+        <v>-0.5</v>
+      </c>
+      <c r="C43" s="4">
+        <f t="shared" si="2"/>
+        <v>45016</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A44">
+        <f t="shared" si="3"/>
+        <v>44987</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C44" s="4" t="e">
+        <f t="shared" ref="C44:C55" si="4">EOMONTH(A44,B44)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A45">
+        <f t="shared" si="3"/>
+        <v>44987</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C45" s="4">
+        <f t="shared" si="4"/>
+        <v>44926</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A46">
+        <f t="shared" si="3"/>
+        <v>44987</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C46" s="4">
+        <f t="shared" si="4"/>
+        <v>45107</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A47" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B47" s="5">
+        <v>1</v>
+      </c>
+      <c r="C47" s="4" t="e">
+        <f t="shared" si="4"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A48" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B48" s="5">
+        <v>1</v>
+      </c>
+      <c r="C48" s="4">
+        <f t="shared" si="4"/>
+        <v>45869</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A49" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B49" s="5">
+        <v>1</v>
+      </c>
+      <c r="C49" s="4">
+        <f t="shared" si="4"/>
+        <v>45046</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A50" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="C50" s="4" t="e">
+        <f t="shared" si="4"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A51" s="1">
+        <f>DATE(2023,3,2)+0.9999999</f>
+        <v>44987.999999899999</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51" s="4">
+        <f t="shared" si="4"/>
+        <v>45046</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A52" s="1">
+        <f>DATE(2023,3,2)+0.5</f>
+        <v>44987.5</v>
+      </c>
+      <c r="B52">
+        <v>0</v>
+      </c>
+      <c r="C52" s="4">
+        <f t="shared" si="4"/>
+        <v>45016</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A53" s="1" t="e">
+        <f>1/0</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53" s="4" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A54" s="1">
+        <f>DATE(2023,3,2)</f>
+        <v>44987</v>
+      </c>
+      <c r="B54" t="e">
+        <f>1/0</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C54" s="4" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A55" s="1" t="e">
+        <f>NA()</f>
+        <v>#N/A</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+      <c r="C55" s="4" t="e">
+        <f t="shared" si="4"/>
+        <v>#N/A</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A56" s="1">
+        <f t="shared" ref="A56:A57" si="5">DATE(2023,3,2)</f>
+        <v>44987</v>
+      </c>
+      <c r="C56" s="4">
+        <f t="shared" ref="C56:C57" si="6">EOMONTH(A56,B56)</f>
+        <v>45016</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.5">
+      <c r="A57" s="1">
+        <f t="shared" si="5"/>
+        <v>44987</v>
+      </c>
+      <c r="C57" s="4">
+        <f t="shared" si="6"/>
+        <v>45016</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>